<commit_message>
fix: integrate Android E2E reports into deploy-and-test workflow and add Web + Android Excel and HTML links to header bar
</commit_message>
<xml_diff>
--- a/Test_Results/Android/android-report.xlsx
+++ b/Test_Results/Android/android-report.xlsx
@@ -7441,7 +7441,7 @@
     <mergeCell ref="A1:B1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -7800,7 +7800,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
 
@@ -33400,6 +33400,6 @@
   </sheetData>
   <autoFilter ref="A1:G1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>
 </file>
</xml_diff>